<commit_message>
Aggiunti esercizi 22 e 23
</commit_message>
<xml_diff>
--- a/Es_11.xlsx
+++ b/Es_11.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon\Documents\Repository\GPOI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{407D06D8-D92C-4031-B844-C8F0532D0203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DAD8253-04C7-48EB-8F58-7F51BDEA54A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
   <si>
     <t>DATI</t>
   </si>
@@ -2054,54 +2054,63 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="C2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="B3" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="C3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="B4" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -2112,7 +2121,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -2123,7 +2132,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>3</v>
       </c>
@@ -2134,12 +2143,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -2150,12 +2159,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>15</v>
       </c>
@@ -2166,12 +2175,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>19</v>
       </c>
@@ -2188,7 +2197,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="7">
         <v>0</v>
       </c>
@@ -2209,7 +2218,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="7">
         <v>1</v>
       </c>
@@ -2230,7 +2239,7 @@
         <v>29.625</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="7">
         <v>2</v>
       </c>
@@ -2251,7 +2260,7 @@
         <v>29.25</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="7">
         <v>3</v>
       </c>
@@ -2272,7 +2281,7 @@
         <v>28.875</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="7">
         <v>4</v>
       </c>
@@ -2293,7 +2302,7 @@
         <v>28.5</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="7">
         <v>5</v>
       </c>
@@ -2314,7 +2323,7 @@
         <v>28.125</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="7">
         <v>6</v>
       </c>
@@ -2332,7 +2341,7 @@
         <v>27.75</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="7">
         <v>7</v>
       </c>
@@ -2350,7 +2359,7 @@
         <v>27.375</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="7">
         <v>8</v>
       </c>
@@ -2368,7 +2377,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="7">
         <v>9</v>
       </c>
@@ -2386,7 +2395,7 @@
         <v>26.625</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="7">
         <v>10</v>
       </c>
@@ -2404,7 +2413,7 @@
         <v>26.25</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="7">
         <v>11</v>
       </c>
@@ -2422,7 +2431,7 @@
         <v>25.875</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="7">
         <v>12</v>
       </c>
@@ -2440,7 +2449,7 @@
         <v>25.5</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="7">
         <v>13</v>
       </c>
@@ -2458,7 +2467,7 @@
         <v>25.125</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="7">
         <v>14</v>
       </c>
@@ -2476,7 +2485,7 @@
         <v>24.75</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="7">
         <v>15</v>
       </c>
@@ -2494,11 +2503,11 @@
         <v>24.375</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
     </row>

</xml_diff>